<commit_message>
Revisión del interventor (MP): seis piezas en el capítulo de modo plan, duraciones de la agenda, tarea sin cuenta de empresa, textos del paso 2, hoja de detalle con nombre neutro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datasets/mp/02 Pedidos por zona y asesora - sintético.xlsx
+++ b/datasets/mp/02 Pedidos por zona y asesora - sintético.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen por zona" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle asesoras Z05 C10" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle asesoras (muestra)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LÉAME" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -11936,7 +11936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -11991,8 +11991,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>